<commit_message>
fix(procesos): corregir guardado Ley Ag y toggle editar/guardar
</commit_message>
<xml_diff>
--- a/INVENTARIO  REPORTE DE INSUMOS CRITICOS (1).xlsx
+++ b/INVENTARIO  REPORTE DE INSUMOS CRITICOS (1).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Desktop\Juan\seguimiento\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Akemi\Documents\Dev\refineria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB83684-FB46-40D8-8999-45647CE1B900}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67ABD3B9-0036-4CE2-8798-A345981E9B41}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C10A7796-865D-4E07-8490-532451BF0998}"/>
   </bookViews>
@@ -29,10 +29,10 @@
         <xcalcf:feature name="microsoft.com:RD"/>
         <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -331,7 +331,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -991,6 +991,57 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -998,57 +1049,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1666,66 +1666,66 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B9DBCA5-C9AD-4F15-86A2-7279E76BA768}">
   <dimension ref="B8:M34"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
-    <col min="2" max="2" width="21.6640625" customWidth="1"/>
+    <col min="2" max="2" width="21.69921875" customWidth="1"/>
     <col min="3" max="4" width="0" hidden="1" customWidth="1"/>
-    <col min="8" max="8" width="17.109375" customWidth="1"/>
-    <col min="10" max="10" width="19.44140625" customWidth="1"/>
-    <col min="13" max="13" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.09765625" customWidth="1"/>
+    <col min="10" max="10" width="19.3984375" customWidth="1"/>
+    <col min="13" max="13" width="12.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="9" spans="2:13" x14ac:dyDescent="0.3">
-      <c r="B9" s="68" t="s">
+    <row r="8" spans="2:13" ht="14.4" thickBot="1"/>
+    <row r="9" spans="2:13">
+      <c r="B9" s="65" t="s">
         <v>27</v>
       </c>
-      <c r="C9" s="69"/>
-      <c r="D9" s="69"/>
-      <c r="E9" s="69"/>
-      <c r="F9" s="69"/>
-      <c r="G9" s="69"/>
-      <c r="H9" s="69"/>
-      <c r="I9" s="69"/>
-      <c r="J9" s="69"/>
-      <c r="K9" s="69"/>
-      <c r="L9" s="69"/>
-      <c r="M9" s="70"/>
-    </row>
-    <row r="10" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B10" s="71"/>
-      <c r="C10" s="72"/>
-      <c r="D10" s="72"/>
-      <c r="E10" s="72"/>
-      <c r="F10" s="72"/>
-      <c r="G10" s="72"/>
-      <c r="H10" s="72"/>
-      <c r="I10" s="72"/>
-      <c r="J10" s="72"/>
-      <c r="K10" s="72"/>
-      <c r="L10" s="72"/>
-      <c r="M10" s="73"/>
-    </row>
-    <row r="17" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="18" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B18" s="77" t="s">
+      <c r="C9" s="66"/>
+      <c r="D9" s="66"/>
+      <c r="E9" s="66"/>
+      <c r="F9" s="66"/>
+      <c r="G9" s="66"/>
+      <c r="H9" s="66"/>
+      <c r="I9" s="66"/>
+      <c r="J9" s="66"/>
+      <c r="K9" s="66"/>
+      <c r="L9" s="66"/>
+      <c r="M9" s="67"/>
+    </row>
+    <row r="10" spans="2:13" ht="14.4" thickBot="1">
+      <c r="B10" s="68"/>
+      <c r="C10" s="69"/>
+      <c r="D10" s="69"/>
+      <c r="E10" s="69"/>
+      <c r="F10" s="69"/>
+      <c r="G10" s="69"/>
+      <c r="H10" s="69"/>
+      <c r="I10" s="69"/>
+      <c r="J10" s="69"/>
+      <c r="K10" s="69"/>
+      <c r="L10" s="69"/>
+      <c r="M10" s="70"/>
+    </row>
+    <row r="17" spans="2:13" ht="14.4" thickBot="1"/>
+    <row r="18" spans="2:13" ht="14.4" thickBot="1">
+      <c r="B18" s="74" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="78"/>
-      <c r="D18" s="78"/>
-      <c r="E18" s="78"/>
-      <c r="F18" s="78"/>
-      <c r="G18" s="78"/>
-      <c r="H18" s="78"/>
-      <c r="J18" s="74" t="s">
+      <c r="C18" s="75"/>
+      <c r="D18" s="75"/>
+      <c r="E18" s="75"/>
+      <c r="F18" s="75"/>
+      <c r="G18" s="75"/>
+      <c r="H18" s="75"/>
+      <c r="J18" s="71" t="s">
         <v>17</v>
       </c>
-      <c r="K18" s="75"/>
-      <c r="L18" s="75"/>
-      <c r="M18" s="76"/>
-    </row>
-    <row r="19" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="20" spans="2:13" ht="55.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K18" s="72"/>
+      <c r="L18" s="72"/>
+      <c r="M18" s="73"/>
+    </row>
+    <row r="19" spans="2:13" ht="14.4" thickBot="1"/>
+    <row r="20" spans="2:13" ht="53.4" thickBot="1">
       <c r="B20" s="26" t="s">
         <v>0</v>
       </c>
@@ -1760,7 +1760,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="21" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:13">
       <c r="B21" s="27" t="s">
         <v>1</v>
       </c>
@@ -1797,7 +1797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:13">
       <c r="B22" s="28" t="s">
         <v>2</v>
       </c>
@@ -1834,7 +1834,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="2:13" ht="14.4" thickBot="1">
       <c r="B23" s="28" t="s">
         <v>3</v>
       </c>
@@ -1871,7 +1871,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:13">
       <c r="B24" s="28" t="s">
         <v>4</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>55.944444444444443</v>
       </c>
     </row>
-    <row r="25" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="2:13">
       <c r="B25" s="28" t="s">
         <v>5</v>
       </c>
@@ -1920,7 +1920,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="2:13">
       <c r="B26" s="28" t="s">
         <v>6</v>
       </c>
@@ -1944,7 +1944,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="27" spans="2:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="2:13">
       <c r="B27" s="28" t="s">
         <v>7</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>5.666666666666667</v>
       </c>
     </row>
-    <row r="28" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:13" ht="14.4" thickBot="1">
       <c r="B28" s="29" t="s">
         <v>8</v>
       </c>
@@ -1994,14 +1994,14 @@
         <v>20</v>
       </c>
     </row>
-    <row r="32" spans="2:13" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="33" spans="10:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="J33" s="66" t="s">
+    <row r="32" spans="2:13" ht="14.4" thickBot="1"/>
+    <row r="33" spans="10:11" ht="14.4" thickBot="1">
+      <c r="J33" s="63" t="s">
         <v>26</v>
       </c>
-      <c r="K33" s="67"/>
-    </row>
-    <row r="34" spans="10:11" ht="23.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="K33" s="64"/>
+    </row>
+    <row r="34" spans="10:11" ht="23.4" customHeight="1" thickBot="1">
       <c r="J34" s="32" t="s">
         <v>23</v>
       </c>
@@ -2025,51 +2025,51 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CCEA64A-F45D-4DC6-8FBC-3D85482A681A}">
   <dimension ref="B4:AK14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
-    <col min="2" max="2" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.8984375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="0" hidden="1" customWidth="1"/>
-    <col min="4" max="29" width="11.5546875" hidden="1" customWidth="1"/>
+    <col min="4" max="29" width="11.59765625" hidden="1" customWidth="1"/>
     <col min="34" max="34" width="0" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:37" x14ac:dyDescent="0.3">
-      <c r="B4" s="79" t="s">
+    <row r="4" spans="2:37">
+      <c r="B4" s="76" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-      <c r="F4" s="79"/>
-      <c r="G4" s="79"/>
-      <c r="H4" s="79"/>
-      <c r="I4" s="79"/>
-      <c r="J4" s="79"/>
-      <c r="K4" s="79"/>
-      <c r="L4" s="79"/>
-      <c r="M4" s="79"/>
-      <c r="N4" s="79"/>
-      <c r="O4" s="79"/>
-      <c r="P4" s="79"/>
-      <c r="Q4" s="79"/>
-      <c r="R4" s="79"/>
-      <c r="S4" s="79"/>
-      <c r="T4" s="79"/>
-      <c r="U4" s="79"/>
-      <c r="V4" s="79"/>
-      <c r="W4" s="79"/>
-      <c r="X4" s="79"/>
-      <c r="Y4" s="79"/>
-      <c r="Z4" s="79"/>
-      <c r="AA4" s="79"/>
-      <c r="AB4" s="79"/>
-      <c r="AC4" s="79"/>
-      <c r="AD4" s="79"/>
-      <c r="AE4" s="79"/>
-      <c r="AF4" s="79"/>
-      <c r="AG4" s="79"/>
-    </row>
-    <row r="6" spans="2:37" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+      <c r="F4" s="76"/>
+      <c r="G4" s="76"/>
+      <c r="H4" s="76"/>
+      <c r="I4" s="76"/>
+      <c r="J4" s="76"/>
+      <c r="K4" s="76"/>
+      <c r="L4" s="76"/>
+      <c r="M4" s="76"/>
+      <c r="N4" s="76"/>
+      <c r="O4" s="76"/>
+      <c r="P4" s="76"/>
+      <c r="Q4" s="76"/>
+      <c r="R4" s="76"/>
+      <c r="S4" s="76"/>
+      <c r="T4" s="76"/>
+      <c r="U4" s="76"/>
+      <c r="V4" s="76"/>
+      <c r="W4" s="76"/>
+      <c r="X4" s="76"/>
+      <c r="Y4" s="76"/>
+      <c r="Z4" s="76"/>
+      <c r="AA4" s="76"/>
+      <c r="AB4" s="76"/>
+      <c r="AC4" s="76"/>
+      <c r="AD4" s="76"/>
+      <c r="AE4" s="76"/>
+      <c r="AF4" s="76"/>
+      <c r="AG4" s="76"/>
+    </row>
+    <row r="6" spans="2:37" ht="41.4" customHeight="1">
       <c r="B6" s="2" t="s">
         <v>0</v>
       </c>
@@ -2167,7 +2167,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="2:37" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:37">
       <c r="B7" s="3" t="s">
         <v>1</v>
       </c>
@@ -2271,7 +2271,7 @@
         <v>1133</v>
       </c>
     </row>
-    <row r="8" spans="2:37" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:37">
       <c r="B8" s="3" t="s">
         <v>2</v>
       </c>
@@ -2378,7 +2378,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="2:37" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:37">
       <c r="B9" s="3" t="s">
         <v>3</v>
       </c>
@@ -2482,7 +2482,7 @@
         <v>4520</v>
       </c>
     </row>
-    <row r="10" spans="2:37" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:37">
       <c r="B10" s="3" t="s">
         <v>4</v>
       </c>
@@ -2586,7 +2586,7 @@
         <v>4028</v>
       </c>
     </row>
-    <row r="11" spans="2:37" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:37">
       <c r="B11" s="3" t="s">
         <v>5</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="12" spans="2:37" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:37">
       <c r="B12" s="3" t="s">
         <v>6</v>
       </c>
@@ -2792,7 +2792,7 @@
         <v>1804</v>
       </c>
     </row>
-    <row r="13" spans="2:37" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:37">
       <c r="B13" s="3" t="s">
         <v>7</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>520</v>
       </c>
     </row>
-    <row r="14" spans="2:37" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:37">
       <c r="B14" s="3" t="s">
         <v>8</v>
       </c>
@@ -3011,20 +3011,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{355AD23F-600D-44E6-834B-F3D31A2B4A17}">
   <dimension ref="B4:E9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
-    <col min="2" max="2" width="11.5546875" customWidth="1"/>
+    <col min="2" max="2" width="11.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:5" x14ac:dyDescent="0.3">
-      <c r="B4" s="79" t="s">
+    <row r="4" spans="2:5">
+      <c r="B4" s="76" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="79"/>
-      <c r="D4" s="79"/>
-      <c r="E4" s="79"/>
-    </row>
-    <row r="6" spans="2:5" x14ac:dyDescent="0.3">
+      <c r="C4" s="76"/>
+      <c r="D4" s="76"/>
+      <c r="E4" s="76"/>
+    </row>
+    <row r="6" spans="2:5">
       <c r="B6" s="2" t="s">
         <v>16</v>
       </c>
@@ -3038,7 +3038,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="7" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:5">
       <c r="B7" s="2" t="s">
         <v>11</v>
       </c>
@@ -3052,7 +3052,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:5">
       <c r="B8" s="2" t="s">
         <v>12</v>
       </c>
@@ -3066,7 +3066,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="2:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:5">
       <c r="B9" s="2" t="s">
         <v>13</v>
       </c>
@@ -3092,22 +3092,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7199A3E2-F429-40A9-984A-C690F6F73EB0}">
   <dimension ref="C3:H70"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
-    <col min="3" max="3" width="23.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="23.69921875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="4" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="C4" s="80" t="s">
+    <row r="3" spans="3:8" ht="14.4" thickBot="1"/>
+    <row r="4" spans="3:8" ht="14.4" thickBot="1">
+      <c r="C4" s="77" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="81"/>
-      <c r="E4" s="82"/>
-    </row>
-    <row r="5" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="6" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="D4" s="78"/>
+      <c r="E4" s="79"/>
+    </row>
+    <row r="5" spans="3:8" ht="14.4" thickBot="1"/>
+    <row r="6" spans="3:8" ht="14.4" thickBot="1">
       <c r="C6" s="4" t="s">
         <v>20</v>
       </c>
@@ -3115,15 +3115,15 @@
         <v>21449</v>
       </c>
     </row>
-    <row r="7" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:8">
       <c r="C7" s="20"/>
       <c r="D7" s="21"/>
     </row>
-    <row r="8" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="3:8" ht="14.4" thickBot="1">
       <c r="C8" s="20"/>
       <c r="D8" s="21"/>
     </row>
-    <row r="9" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="3:8" ht="14.4" thickBot="1">
       <c r="C9" s="22" t="s">
         <v>23</v>
       </c>
@@ -3132,12 +3132,12 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="10" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:8">
       <c r="C10" s="20"/>
       <c r="D10" s="21"/>
     </row>
-    <row r="11" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="12" spans="3:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="3:8" ht="14.4" thickBot="1"/>
+    <row r="12" spans="3:8" ht="14.4" thickBot="1">
       <c r="C12" s="5" t="s">
         <v>21</v>
       </c>
@@ -3148,7 +3148,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="13" spans="3:8">
       <c r="C13" s="40">
         <v>46174</v>
       </c>
@@ -3164,7 +3164,7 @@
         <v>-3000</v>
       </c>
     </row>
-    <row r="14" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="14" spans="3:8">
       <c r="C14" s="14">
         <v>46175</v>
       </c>
@@ -3176,7 +3176,7 @@
         <v>18036</v>
       </c>
     </row>
-    <row r="15" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:8">
       <c r="C15" s="14">
         <v>46175</v>
       </c>
@@ -3188,7 +3188,7 @@
         <v>17976</v>
       </c>
     </row>
-    <row r="16" spans="3:8" x14ac:dyDescent="0.3">
+    <row r="16" spans="3:8">
       <c r="C16" s="14">
         <v>46178</v>
       </c>
@@ -3200,7 +3200,7 @@
         <v>15926</v>
       </c>
     </row>
-    <row r="17" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="3:5">
       <c r="C17" s="14">
         <v>46181</v>
       </c>
@@ -3212,7 +3212,7 @@
         <v>13880</v>
       </c>
     </row>
-    <row r="18" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="3:5">
       <c r="C18" s="14">
         <v>46186</v>
       </c>
@@ -3224,7 +3224,7 @@
         <v>12880</v>
       </c>
     </row>
-    <row r="19" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:5">
       <c r="C19" s="14">
         <v>46188</v>
       </c>
@@ -3236,7 +3236,7 @@
         <v>11880</v>
       </c>
     </row>
-    <row r="20" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:5">
       <c r="C20" s="14">
         <v>46192</v>
       </c>
@@ -3248,7 +3248,7 @@
         <v>8067</v>
       </c>
     </row>
-    <row r="21" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="3:5">
       <c r="C21" s="14">
         <v>46194</v>
       </c>
@@ -3260,7 +3260,7 @@
         <v>7067</v>
       </c>
     </row>
-    <row r="22" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:5">
       <c r="C22" s="14">
         <v>46196</v>
       </c>
@@ -3272,7 +3272,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="23" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="3:5">
       <c r="C23" s="10"/>
       <c r="D23" s="11"/>
       <c r="E23" s="12">
@@ -3280,7 +3280,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="24" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="3:5">
       <c r="C24" s="10"/>
       <c r="D24" s="11"/>
       <c r="E24" s="12">
@@ -3288,7 +3288,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="25" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="3:5">
       <c r="C25" s="10"/>
       <c r="D25" s="11"/>
       <c r="E25" s="12">
@@ -3296,7 +3296,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="26" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="26" spans="3:5">
       <c r="C26" s="10"/>
       <c r="D26" s="11"/>
       <c r="E26" s="12">
@@ -3304,7 +3304,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="27" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="27" spans="3:5">
       <c r="C27" s="10"/>
       <c r="D27" s="11"/>
       <c r="E27" s="12">
@@ -3312,7 +3312,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="28" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="28" spans="3:5">
       <c r="C28" s="10"/>
       <c r="D28" s="11"/>
       <c r="E28" s="12">
@@ -3320,7 +3320,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="29" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="29" spans="3:5">
       <c r="C29" s="10"/>
       <c r="D29" s="11"/>
       <c r="E29" s="12">
@@ -3328,7 +3328,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="30" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:5">
       <c r="C30" s="10"/>
       <c r="D30" s="11"/>
       <c r="E30" s="12">
@@ -3336,7 +3336,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="31" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="31" spans="3:5">
       <c r="C31" s="10"/>
       <c r="D31" s="11"/>
       <c r="E31" s="13">
@@ -3344,7 +3344,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="32" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="32" spans="3:5">
       <c r="C32" s="10"/>
       <c r="D32" s="11"/>
       <c r="E32" s="13">
@@ -3352,7 +3352,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="33" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="33" spans="3:5">
       <c r="C33" s="10"/>
       <c r="D33" s="11"/>
       <c r="E33" s="13">
@@ -3360,7 +3360,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="34" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="34" spans="3:5">
       <c r="C34" s="10"/>
       <c r="D34" s="11"/>
       <c r="E34" s="13">
@@ -3368,7 +3368,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="35" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="35" spans="3:5">
       <c r="C35" s="10"/>
       <c r="D35" s="11"/>
       <c r="E35" s="13">
@@ -3376,7 +3376,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="36" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="36" spans="3:5">
       <c r="C36" s="10"/>
       <c r="D36" s="11"/>
       <c r="E36" s="13">
@@ -3384,7 +3384,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="37" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="37" spans="3:5">
       <c r="C37" s="10"/>
       <c r="D37" s="11"/>
       <c r="E37" s="13">
@@ -3392,7 +3392,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="38" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="38" spans="3:5">
       <c r="C38" s="10"/>
       <c r="D38" s="11"/>
       <c r="E38" s="13">
@@ -3400,7 +3400,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="39" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="39" spans="3:5">
       <c r="C39" s="10"/>
       <c r="D39" s="11"/>
       <c r="E39" s="13">
@@ -3408,7 +3408,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="40" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="40" spans="3:5">
       <c r="C40" s="14"/>
       <c r="D40" s="11"/>
       <c r="E40" s="13">
@@ -3416,7 +3416,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="41" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="41" spans="3:5">
       <c r="C41" s="14"/>
       <c r="D41" s="11"/>
       <c r="E41" s="13">
@@ -3424,7 +3424,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="42" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="42" spans="3:5">
       <c r="C42" s="14"/>
       <c r="D42" s="11"/>
       <c r="E42" s="13">
@@ -3432,7 +3432,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="43" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="43" spans="3:5">
       <c r="C43" s="14"/>
       <c r="D43" s="11"/>
       <c r="E43" s="13">
@@ -3440,7 +3440,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="44" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="44" spans="3:5">
       <c r="C44" s="14"/>
       <c r="D44" s="11"/>
       <c r="E44" s="13">
@@ -3448,7 +3448,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="45" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="45" spans="3:5">
       <c r="C45" s="14"/>
       <c r="D45" s="11"/>
       <c r="E45" s="13">
@@ -3456,7 +3456,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="46" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="46" spans="3:5">
       <c r="C46" s="14"/>
       <c r="D46" s="11"/>
       <c r="E46" s="13">
@@ -3464,7 +3464,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="47" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="47" spans="3:5">
       <c r="C47" s="14"/>
       <c r="D47" s="11"/>
       <c r="E47" s="13">
@@ -3472,7 +3472,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="48" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="48" spans="3:5">
       <c r="C48" s="14"/>
       <c r="D48" s="11"/>
       <c r="E48" s="13">
@@ -3480,7 +3480,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="49" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="49" spans="3:5">
       <c r="C49" s="14"/>
       <c r="D49" s="11"/>
       <c r="E49" s="13">
@@ -3488,7 +3488,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="50" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="50" spans="3:5">
       <c r="C50" s="14"/>
       <c r="D50" s="11"/>
       <c r="E50" s="13">
@@ -3496,7 +3496,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="51" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="51" spans="3:5">
       <c r="C51" s="14"/>
       <c r="D51" s="11"/>
       <c r="E51" s="13">
@@ -3504,7 +3504,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="52" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="52" spans="3:5">
       <c r="C52" s="14"/>
       <c r="D52" s="11"/>
       <c r="E52" s="13">
@@ -3512,7 +3512,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="53" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="53" spans="3:5">
       <c r="C53" s="14"/>
       <c r="D53" s="11"/>
       <c r="E53" s="13">
@@ -3520,7 +3520,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="54" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="54" spans="3:5">
       <c r="C54" s="14"/>
       <c r="D54" s="11"/>
       <c r="E54" s="13">
@@ -3528,7 +3528,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="55" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="55" spans="3:5">
       <c r="C55" s="14"/>
       <c r="D55" s="11"/>
       <c r="E55" s="13">
@@ -3536,7 +3536,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="56" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="56" spans="3:5">
       <c r="C56" s="14"/>
       <c r="D56" s="11"/>
       <c r="E56" s="13">
@@ -3544,7 +3544,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="57" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="57" spans="3:5">
       <c r="C57" s="14"/>
       <c r="D57" s="15"/>
       <c r="E57" s="13">
@@ -3552,7 +3552,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="58" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="58" spans="3:5">
       <c r="C58" s="14"/>
       <c r="D58" s="11"/>
       <c r="E58" s="13">
@@ -3560,7 +3560,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="59" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="59" spans="3:5">
       <c r="C59" s="10"/>
       <c r="D59" s="11"/>
       <c r="E59" s="13">
@@ -3568,7 +3568,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="60" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="60" spans="3:5">
       <c r="C60" s="10"/>
       <c r="D60" s="11"/>
       <c r="E60" s="13">
@@ -3576,7 +3576,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="61" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="61" spans="3:5">
       <c r="C61" s="10"/>
       <c r="D61" s="11"/>
       <c r="E61" s="13">
@@ -3584,7 +3584,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="62" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="62" spans="3:5">
       <c r="C62" s="10"/>
       <c r="D62" s="11"/>
       <c r="E62" s="13">
@@ -3592,7 +3592,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="63" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="63" spans="3:5">
       <c r="C63" s="10"/>
       <c r="D63" s="11"/>
       <c r="E63" s="13">
@@ -3600,7 +3600,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="64" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="64" spans="3:5">
       <c r="C64" s="10"/>
       <c r="D64" s="11"/>
       <c r="E64" s="13">
@@ -3608,7 +3608,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="65" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="65" spans="3:5">
       <c r="C65" s="10"/>
       <c r="D65" s="11"/>
       <c r="E65" s="13">
@@ -3616,7 +3616,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="66" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="66" spans="3:5">
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="13">
@@ -3624,7 +3624,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="67" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="67" spans="3:5">
       <c r="C67" s="10"/>
       <c r="D67" s="11"/>
       <c r="E67" s="13">
@@ -3632,7 +3632,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="68" spans="3:5" x14ac:dyDescent="0.3">
+    <row r="68" spans="3:5">
       <c r="C68" s="10"/>
       <c r="D68" s="11"/>
       <c r="E68" s="13">
@@ -3640,7 +3640,7 @@
         <v>5067</v>
       </c>
     </row>
-    <row r="69" spans="3:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="69" spans="3:5" ht="14.4" thickBot="1">
       <c r="C69" s="16" t="s">
         <v>24</v>
       </c>
@@ -3650,7 +3650,7 @@
       </c>
       <c r="E69" s="1"/>
     </row>
-    <row r="70" spans="3:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="3:5" ht="14.4" thickBot="1">
       <c r="C70" s="18" t="s">
         <v>25</v>
       </c>
@@ -3671,56 +3671,56 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E165D15B-641B-4CED-8D93-58C054B5A031}">
   <dimension ref="B1:D14"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
-    <col min="2" max="2" width="31.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.44140625" customWidth="1"/>
+    <col min="2" max="2" width="31.19921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.3984375" customWidth="1"/>
     <col min="4" max="4" width="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:4">
       <c r="B1" s="50"/>
       <c r="C1" s="50"/>
       <c r="D1" s="50"/>
     </row>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4">
       <c r="B2" s="50"/>
       <c r="C2" s="50"/>
       <c r="D2" s="50"/>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4">
       <c r="B3" s="50"/>
       <c r="C3" s="50"/>
       <c r="D3" s="50"/>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4">
       <c r="B4" s="50"/>
       <c r="C4" s="50"/>
       <c r="D4" s="50"/>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4">
       <c r="B5" s="50"/>
       <c r="C5" s="50"/>
       <c r="D5" s="50"/>
     </row>
-    <row r="6" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="2:4" ht="14.4" thickBot="1">
       <c r="B6" s="50"/>
       <c r="C6" s="50"/>
       <c r="D6" s="50"/>
     </row>
-    <row r="7" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="63" t="s">
+    <row r="7" spans="2:4" ht="14.4" thickBot="1">
+      <c r="B7" s="80" t="s">
         <v>32</v>
       </c>
-      <c r="C7" s="64"/>
-      <c r="D7" s="65"/>
-    </row>
-    <row r="8" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="C7" s="81"/>
+      <c r="D7" s="82"/>
+    </row>
+    <row r="8" spans="2:4" ht="14.4" thickBot="1">
       <c r="B8" s="50"/>
       <c r="C8" s="50"/>
       <c r="D8" s="50"/>
     </row>
-    <row r="9" spans="2:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="2:4" ht="14.4" thickBot="1">
       <c r="B9" s="51" t="s">
         <v>29</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="115.8" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="2:4" ht="111" thickBot="1">
       <c r="B10" s="45" t="s">
         <v>48</v>
       </c>
@@ -3742,7 +3742,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="2:4" ht="28.2" thickBot="1">
       <c r="B11" s="58" t="s">
         <v>74</v>
       </c>
@@ -3753,7 +3753,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="72" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:4" ht="69">
       <c r="B12" s="45" t="s">
         <v>49</v>
       </c>
@@ -3764,7 +3764,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="46.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="2:4" ht="46.2" customHeight="1" thickBot="1">
       <c r="B13" s="54" t="s">
         <v>40</v>
       </c>
@@ -3775,7 +3775,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4">
       <c r="B14" s="50"/>
       <c r="C14" s="50"/>
       <c r="D14" s="50"/>

</xml_diff>